<commit_message>
Created the DataProviderUtil for the Excel data that is used in the createJobAPITest
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PhoenixTestData.xlsx
+++ b/src/test/resources/testData/PhoenixTestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LoginTestData" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="54">
   <si>
     <t>username</t>
   </si>
@@ -35,6 +35,153 @@
   </si>
   <si>
     <t>iameng</t>
+  </si>
+  <si>
+    <t>mst_service_location_id</t>
+  </si>
+  <si>
+    <t>mst_platform_id</t>
+  </si>
+  <si>
+    <t>mst_warrenty_status_id</t>
+  </si>
+  <si>
+    <t>mst_oem_id</t>
+  </si>
+  <si>
+    <t>customer__first_name</t>
+  </si>
+  <si>
+    <t>customer__last_name</t>
+  </si>
+  <si>
+    <t>customer__mobile_number</t>
+  </si>
+  <si>
+    <t>customer__mobile_number_alt</t>
+  </si>
+  <si>
+    <t>customer__email_id</t>
+  </si>
+  <si>
+    <t>customer__email_id_alt</t>
+  </si>
+  <si>
+    <t>customer_address__flat_number</t>
+  </si>
+  <si>
+    <t>customer_address__apartment_name</t>
+  </si>
+  <si>
+    <t>customer_address__street_name</t>
+  </si>
+  <si>
+    <t>customer_address__landmark</t>
+  </si>
+  <si>
+    <t>customer_address__area</t>
+  </si>
+  <si>
+    <t>customer_address__pincode</t>
+  </si>
+  <si>
+    <t>customer_address__country</t>
+  </si>
+  <si>
+    <t>customer_address__state</t>
+  </si>
+  <si>
+    <t>customer_product__dop</t>
+  </si>
+  <si>
+    <t>customer_product__serial_number</t>
+  </si>
+  <si>
+    <t>customer_product__imei1</t>
+  </si>
+  <si>
+    <t>customer_product__imei2</t>
+  </si>
+  <si>
+    <t>customer_product__popurl</t>
+  </si>
+  <si>
+    <t>customer_product__product_id</t>
+  </si>
+  <si>
+    <t>customer_product__mst_model_id</t>
+  </si>
+  <si>
+    <t>problems__id</t>
+  </si>
+  <si>
+    <t>problems__remark</t>
+  </si>
+  <si>
+    <t>Darrel</t>
+  </si>
+  <si>
+    <t>Abernathy</t>
+  </si>
+  <si>
+    <t>948-272-7422</t>
+  </si>
+  <si>
+    <t>Julius_Beatty65@yahoo.com</t>
+  </si>
+  <si>
+    <t>c 304</t>
+  </si>
+  <si>
+    <t>Jupiter</t>
+  </si>
+  <si>
+    <t>MG road</t>
+  </si>
+  <si>
+    <t>Bangur Nagar</t>
+  </si>
+  <si>
+    <t>Goregaon West</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Maharashtra</t>
+  </si>
+  <si>
+    <t>2025-04-06T18:30:00.000Z</t>
+  </si>
+  <si>
+    <t>Battery Issue</t>
+  </si>
+  <si>
+    <t>Sam</t>
+  </si>
+  <si>
+    <t>Joy</t>
+  </si>
+  <si>
+    <t>Niel</t>
+  </si>
+  <si>
+    <t>36885242743732</t>
+  </si>
+  <si>
+    <t>37885242743731</t>
+  </si>
+  <si>
+    <t>46885242743732</t>
+  </si>
+  <si>
+    <t>57885242743731</t>
+  </si>
+  <si>
+    <t>948-272-7423</t>
+  </si>
+  <si>
+    <t>Julius_Beatty35@yahoo.com</t>
   </si>
 </sst>
 </file>
@@ -82,9 +229,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -412,9 +561,456 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="28" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O1" t="s">
+        <v>19</v>
+      </c>
+      <c r="P1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>21</v>
+      </c>
+      <c r="R1" t="s">
+        <v>22</v>
+      </c>
+      <c r="S1" t="s">
+        <v>23</v>
+      </c>
+      <c r="T1" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" t="s">
+        <v>25</v>
+      </c>
+      <c r="V1" t="s">
+        <v>26</v>
+      </c>
+      <c r="W1" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P2">
+        <v>411039</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>41</v>
+      </c>
+      <c r="R2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S2" t="s">
+        <v>43</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="W2" t="s">
+        <v>43</v>
+      </c>
+      <c r="X2">
+        <v>1</v>
+      </c>
+      <c r="Y2">
+        <v>1</v>
+      </c>
+      <c r="Z2">
+        <v>1</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" t="s">
+        <v>53</v>
+      </c>
+      <c r="K3" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" t="s">
+        <v>40</v>
+      </c>
+      <c r="P3">
+        <v>411039</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>41</v>
+      </c>
+      <c r="R3" t="s">
+        <v>42</v>
+      </c>
+      <c r="S3" t="s">
+        <v>43</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="W3" t="s">
+        <v>43</v>
+      </c>
+      <c r="X3">
+        <v>1</v>
+      </c>
+      <c r="Y3">
+        <v>1</v>
+      </c>
+      <c r="Z3">
+        <v>1</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>0</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" t="s">
+        <v>53</v>
+      </c>
+      <c r="K4" t="s">
+        <v>36</v>
+      </c>
+      <c r="L4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" t="s">
+        <v>39</v>
+      </c>
+      <c r="O4" t="s">
+        <v>40</v>
+      </c>
+      <c r="P4">
+        <v>411039</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>41</v>
+      </c>
+      <c r="R4" t="s">
+        <v>42</v>
+      </c>
+      <c r="S4" t="s">
+        <v>43</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="W4" t="s">
+        <v>43</v>
+      </c>
+      <c r="X4">
+        <v>1</v>
+      </c>
+      <c r="Y4">
+        <v>1</v>
+      </c>
+      <c r="Z4">
+        <v>1</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>0</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" t="s">
+        <v>53</v>
+      </c>
+      <c r="K5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L5" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O5" t="s">
+        <v>40</v>
+      </c>
+      <c r="P5">
+        <v>411039</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>41</v>
+      </c>
+      <c r="R5" t="s">
+        <v>42</v>
+      </c>
+      <c r="S5" t="s">
+        <v>43</v>
+      </c>
+      <c r="T5" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="U5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="W5" t="s">
+        <v>43</v>
+      </c>
+      <c r="X5">
+        <v>1</v>
+      </c>
+      <c r="Y5">
+        <v>1</v>
+      </c>
+      <c r="Z5">
+        <v>1</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>